<commit_message>
File changes and readme update
</commit_message>
<xml_diff>
--- a/EnergyPrices and Supporting Data/2014Prices/Energy Rates_2014.xlsx
+++ b/EnergyPrices and Supporting Data/2014Prices/Energy Rates_2014.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="57510" yWindow="-90" windowWidth="23235" windowHeight="12555"/>
+    <workbookView xWindow="57510" yWindow="-90" windowWidth="23235" windowHeight="12555" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="April" sheetId="5" r:id="rId1"/>
@@ -1309,7 +1309,6 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -1615,7 +1614,6 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
@@ -2439,7 +2437,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US" sz="1600" b="1"/>
-              <a:t>Prize (August</a:t>
+              <a:t>Price (August</a:t>
             </a:r>
             <a:r>
               <a:rPr lang="en-US" sz="1600" b="1" baseline="0"/>
@@ -2449,6 +2447,7 @@
           </a:p>
         </c:rich>
       </c:tx>
+      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -2748,6 +2747,7 @@
               </a:p>
             </c:rich>
           </c:tx>
+          <c:layout/>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
@@ -2978,6 +2978,7 @@
           </a:p>
         </c:rich>
       </c:tx>
+      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -3299,6 +3300,7 @@
               </a:p>
             </c:rich>
           </c:tx>
+          <c:layout/>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
@@ -3417,6 +3419,7 @@
               </a:p>
             </c:rich>
           </c:tx>
+          <c:layout/>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
@@ -4666,7 +4669,6 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -4976,7 +4978,6 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>

</xml_diff>